<commit_message>
chore(samples): add a second sheet to the xlsx sample for the sheet picker [P3-T3.18]
"Borrowers" stays first (the default), so expected totals don't change;
"Old loans" (2 rows) lets the E2E suite switch sheets.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/samples/contacts-sample-100.xlsx
+++ b/docs/samples/contacts-sample-100.xlsx
@@ -7,6 +7,7 @@
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="Borrowers"/>
+    <sheet r:id="rId2" sheetId="2" name="Old loans"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -1868,6 +1869,24 @@
   </si>
   <si>
     <t>30000</t>
+  </si>
+  <si>
+    <t>Old Borrower 1</t>
+  </si>
+  <si>
+    <t>9000400001</t>
+  </si>
+  <si>
+    <t>1500</t>
+  </si>
+  <si>
+    <t>Old Borrower 2</t>
+  </si>
+  <si>
+    <t>9000400002</t>
+  </si>
+  <si>
+    <t>2500</t>
   </si>
 </sst>
 </file>
@@ -4355,4 +4374,44 @@
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>618</v>
+      </c>
+      <c r="B2" t="s">
+        <v>619</v>
+      </c>
+      <c r="C2" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>621</v>
+      </c>
+      <c r="B3" t="s">
+        <v>622</v>
+      </c>
+      <c r="C3" t="s">
+        <v>623</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>